<commit_message>
fix and update REF
</commit_message>
<xml_diff>
--- a/CargarTransaccionesV2/Data/Input/BaseCambios.xlsx
+++ b/CargarTransaccionesV2/Data/Input/BaseCambios.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0179535F-67D4-4F7B-A7EF-51595A449A8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C973CE64-EA2B-4258-AF4D-0B45DC0B927F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="9">
   <si>
     <t>IdTransaccion</t>
   </si>
@@ -399,6 +399,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -472,9 +475,6 @@
       <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="C5">
-        <v>136.19999999999999</v>
-      </c>
       <c r="D5" t="s">
         <v>8</v>
       </c>
@@ -571,9 +571,6 @@
       <c r="A11">
         <v>10</v>
       </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
       <c r="C11">
         <v>50.25</v>
       </c>
@@ -664,9 +661,6 @@
       </c>
       <c r="D16" t="s">
         <v>8</v>
-      </c>
-      <c r="E16">
-        <v>114.91</v>
       </c>
     </row>
     <row r="17" spans="1:5">

</xml_diff>

<commit_message>
fix condition of queues and to or status
</commit_message>
<xml_diff>
--- a/CargarTransaccionesV2/Data/Input/BaseCambios.xlsx
+++ b/CargarTransaccionesV2/Data/Input/BaseCambios.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C973CE64-EA2B-4258-AF4D-0B45DC0B927F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D3862F0E-3E0C-4CCE-8F58-35DBCBC2CE51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="11">
   <si>
     <t>IdTransaccion</t>
   </si>
@@ -58,6 +58,12 @@
   </si>
   <si>
     <t>MXN</t>
+  </si>
+  <si>
+    <t>AUD</t>
+  </si>
+  <si>
+    <t>ARS</t>
   </si>
 </sst>
 </file>
@@ -620,16 +626,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>243.12</v>
       </c>
       <c r="D14" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E14">
-        <v>243.12</v>
+        <v>243384</v>
       </c>
     </row>
     <row r="15" spans="1:5">

</xml_diff>